<commit_message>
UBAH FORMAT IMPORT DAN EXPORT DENGAN FILTER KOREKSI
</commit_message>
<xml_diff>
--- a/public/format_import/format_import_koreksi_potongan.xlsx
+++ b/public/format_import/format_import_koreksi_potongan.xlsx
@@ -1,30 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andri M\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\hris\public\format_import\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D927A045-BC10-4F8C-B6D0-7E4222DC0450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7530"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
   <si>
     <t>enroll_id</t>
   </si>
@@ -71,29 +83,41 @@
     <t>periode_tanggal_akhir</t>
   </si>
   <si>
-    <t>1. BPJS TK</t>
-  </si>
-  <si>
-    <t>2. BPJS KS</t>
-  </si>
-  <si>
-    <t>3. Bazzar</t>
-  </si>
-  <si>
-    <t>4. Kas Bon</t>
-  </si>
-  <si>
-    <t>5. Lain-lain</t>
+    <t>POTONGAN BPJS TK</t>
+  </si>
+  <si>
+    <t>POTONGAN BPJS KS</t>
+  </si>
+  <si>
+    <t>POTONGAN BAZAR</t>
+  </si>
+  <si>
+    <t>POTONGAN KAS BON</t>
+  </si>
+  <si>
+    <t>POTONGAN LAINNYA</t>
+  </si>
+  <si>
+    <t>POTONGAN KARYAWAN</t>
+  </si>
+  <si>
+    <t>POTONGAN UPAH</t>
+  </si>
+  <si>
+    <t>POTONGAN LEMBUR</t>
+  </si>
+  <si>
+    <t>tanggal_koreksi</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd\-mm\-yyyy"/>
+    <numFmt numFmtId="169" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -104,15 +128,22 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFD4D4D4"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Consolas"/>
-      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -135,17 +166,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -426,8 +460,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:L10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -436,10 +470,13 @@
     <col min="5" max="5" width="19.7109375" customWidth="1"/>
     <col min="6" max="6" width="23.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.42578125" customWidth="1"/>
+    <col min="9" max="9" width="20.28515625" customWidth="1"/>
+    <col min="10" max="10" width="26.140625" customWidth="1"/>
+    <col min="12" max="12" width="29.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -464,8 +501,14 @@
       <c r="H1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>3097</v>
       </c>
@@ -478,23 +521,26 @@
       <c r="D2">
         <v>1000</v>
       </c>
-      <c r="E2" s="2">
-        <v>44952</v>
-      </c>
-      <c r="F2" s="3">
-        <v>44982</v>
+      <c r="E2" s="4">
+        <v>45864</v>
+      </c>
+      <c r="F2" s="5">
+        <v>45894</v>
       </c>
       <c r="G2" t="s">
         <v>9</v>
       </c>
-      <c r="H2">
-        <v>3</v>
+      <c r="H2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="4">
+        <v>45866</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>11</v>
       </c>
@@ -507,41 +553,67 @@
       <c r="D3">
         <v>2000</v>
       </c>
-      <c r="E3" s="2">
-        <v>44952</v>
-      </c>
-      <c r="F3" s="3">
-        <v>44982</v>
+      <c r="E3" s="4">
+        <v>45864</v>
+      </c>
+      <c r="F3" s="5">
+        <v>45894</v>
       </c>
       <c r="G3" t="s">
         <v>12</v>
       </c>
-      <c r="H3">
-        <v>3</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="J4" s="4" t="s">
+      <c r="H3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" s="4">
+        <v>45867</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="J5" s="4" t="s">
+      <c r="L3" s="2"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I4" s="4"/>
+      <c r="J4" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="J6" s="4" t="s">
+      <c r="L4" s="2"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I5" s="4"/>
+      <c r="J5" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="J7" s="4" t="s">
+      <c r="L5" s="2"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J6" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="L6" s="2"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L7" s="2"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="L8" s="2"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="L9" s="2"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J10" s="1"/>
+      <c r="L10" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>